<commit_message>
Add debug logging to diagnose packet storage issue in RunContext
Co-authored-by: dongnuc <136960214+dongnuc@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/batchstudent/Results/StudentsSolution.xlsx
+++ b/batchstudent/Results/StudentsSolution.xlsx
@@ -44,18 +44,6 @@
   </x:si>
   <x:si>
     <x:t/>
-  </x:si>
-  <x:si>
-    <x:t>anlpvhe187047</x:t>
-  </x:si>
-  <x:si>
-    <x:t>cuongnvhe181200</x:t>
-  </x:si>
-  <x:si>
-    <x:t>dungdvhe181404</x:t>
-  </x:si>
-  <x:si>
-    <x:t>dungtdhe186461</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -421,10 +409,10 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:F6"/>
+  <x:dimension ref="A1:F2"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="17.424911" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="15.424911" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="5.996339" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="6.853482" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="10.139196" style="0" customWidth="1"/>
@@ -472,86 +460,6 @@
         <x:v>9</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" spans="1:6">
-      <x:c r="A3" s="0" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="B3" s="0" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C3" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="D3" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E3" s="0">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="F3" s="0" t="s">
-        <x:v>9</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:6">
-      <x:c r="A4" s="0" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B4" s="0" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C4" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="D4" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E4" s="0">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="F4" s="0" t="s">
-        <x:v>9</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:6">
-      <x:c r="A5" s="0" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B5" s="0" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C5" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="D5" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E5" s="0">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="F5" s="0" t="s">
-        <x:v>9</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:6">
-      <x:c r="A6" s="0" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B6" s="0" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C6" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="D6" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E6" s="0">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="F6" s="0" t="s">
-        <x:v>9</x:v>
-      </x:c>
-    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>